<commit_message>
fix(g3-pagemap): apply teacher review fixes on p.100 (2047 blocks) & p.130 (6 bottles, full table)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/authoring/PAGE-MAP-KH-G3-MATH-v1_verified.xlsx
+++ b/authoring/PAGE-MAP-KH-G3-MATH-v1_verified.xlsx
@@ -8093,12 +8093,12 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>تعیین تکلیف هم‌پوشانی: (۱) عنوان بنر اصلی درس در وسط-بالا «مقایسه‌ی عددها» + تاب «فعّالیت» در راست چاپ شده است (در نقشه فقط «فعّالیت» آمده). (۲) تأیید تصویری ۱ـ: بلوک‌های پایهٔ ده عدد ۲۱۱۱ (چپ) و ۲۰۵۵ (راست) را نشان می‌دهند؛ تعداد تمرین شماره‌دار = ۳ (۱ـ تا ۳ـ) صحیح است.</t>
+          <t>تعیین تکلیف هم‌پوشانی: وسط-بالا بنر مستقل درس «مقایسه‌ی عددها» + تاب راست «فعّالیت» با ۳ تمرین شماره‌دار (۱ـ تا ۳ـ) چاپ شده است؛ در شکل ۱ـ بلوک‌های پایهٔ ده چپ نمایندهٔ ۲۱۱۱ و راست نمایندهٔ ۲۰۴۷ (۲ مکعب هزارتایی + ۰ صدتایی + ۴ میلهٔ ده‌تایی + ۷ یکان شامل ۳ ردیف ۲تایی و ۱ تکی بالا-چپ) است.</t>
         </is>
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t>C305.pdf#p=100 — بنر نارنجی وسط-بالا «مقایسه‌ی عددها» + شماره‌های ۱ـ تا ۳ـ</t>
+          <t>C305.pdf#p=100 — بنر نارنجی وسط-بالا «مقایسه‌ی عددها» + فعّالیت ۱ـ تا ۳ـ (بلوک‌های ۲۱۱۱ چپ و ۲۰۴۷ راست)</t>
         </is>
       </c>
     </row>
@@ -10313,12 +10313,12 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>تعیین تکلیف هم‌پوشانی: خوانش G1 (بنر «مرور فصل»، نوع «مرور فصل»، تعداد تمرین شماره‌دار = ۳ شامل فرهنگ نوشتن ۱ـ و ۲ـ و تمرین ۱ـ) کاملاً صحیح است؛ جدول فروش ۶روزه (شنبه=۳۰، یک‌شنبه=۲۵، دوشنبه=۳۵، سه‌شنبه=۱۵، چهارشنبه=۳۰، پنج‌شنبه=۴۰) تماماً پُر و بدون خانهٔ خالی است و سبد پایین-چپ دقیقاً ۶ بطری شیر (۲ ردیف ۳تایی پُر) دارد.</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>C305.pdf#p=130 — تعیین تکلیف هم‌پوشانی: بنر «مرور فصل»، نوع «مرور فصل» و تعداد تمرین شماره‌دار = ۳ (فرهنگ نوشتن ۱ـ و ۲ـ + تمرین ۱ـ جدول شیر؛ ۵ بطری در سبد تصویر) کاملاً صحیح است</t>
+          <t>C305.pdf#p=130 — بنر «مرور فصل» + فرهنگ نوشتن (۱ـ، ۲ـ) + تمرین ۱ـ (جدول ۶روزهٔ پُر + سبد ۶ بطری شیر)</t>
         </is>
       </c>
     </row>

</xml_diff>